<commit_message>
First part of task for NarrativeHint functional. Alex Pavlenko.
</commit_message>
<xml_diff>
--- a/UploadTemplates/addQuestionnaireTemplate.xlsx
+++ b/UploadTemplates/addQuestionnaireTemplate.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Page</t>
   </si>
@@ -126,13 +126,16 @@
   </si>
   <si>
     <t>SubCheckBoxChoice</t>
+  </si>
+  <si>
+    <t>NarrativeHint</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="宋体"/>
@@ -155,6 +158,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="5">
@@ -195,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -231,6 +240,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -619,7 +631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AC1"/>
   <sheetFormatPr defaultColWidth="10.28515625" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="6.5703125" style="7" bestFit="1" customWidth="1"/>
@@ -649,7 +661,7 @@
     <col min="25" max="16384" width="10.28515625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28">
+    <row r="1" spans="1:29">
       <c r="A1" s="3" t="s">
         <v>14</v>
       </c>
@@ -733,6 +745,9 @@
       </c>
       <c r="AB1" s="13" t="s">
         <v>27</v>
+      </c>
+      <c r="AC1" s="14" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>